<commit_message>
Deploying to gh-pages from  @ ea5c5a5b4e08b0af0807aeab04967d895b1088ef 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/GLIDENumber.xlsx
+++ b/api/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14423" uniqueCount="7216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14427" uniqueCount="7218">
   <si>
     <t>code</t>
   </si>
@@ -41,6 +41,12 @@
   </si>
   <si>
     <t>en</t>
+  </si>
+  <si>
+    <t>TC-2020-000238-FJI</t>
+  </si>
+  <si>
+    <t>FL-2020-000237-LKA</t>
   </si>
   <si>
     <t>VO-2020-000236-IDN</t>
@@ -21993,7 +21999,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7209"/>
+  <dimension ref="A1:G7211"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -79683,6 +79689,22 @@
         <v>8</v>
       </c>
     </row>
+    <row r="7210" spans="1:4">
+      <c r="A7210" t="s">
+        <v>7216</v>
+      </c>
+      <c r="D7210" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7211" spans="1:4">
+      <c r="A7211" t="s">
+        <v>7217</v>
+      </c>
+      <c r="D7211" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 946ff8060a18c984ecd7d79ea596591f73a3efce 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/GLIDENumber.xlsx
+++ b/api/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14427" uniqueCount="7218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14429" uniqueCount="7219">
   <si>
     <t>code</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>en</t>
+  </si>
+  <si>
+    <t>TC-2020-000239-MDG</t>
   </si>
   <si>
     <t>TC-2020-000238-FJI</t>
@@ -21999,7 +22002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7211"/>
+  <dimension ref="A1:G7212"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -79705,6 +79708,14 @@
         <v>8</v>
       </c>
     </row>
+    <row r="7212" spans="1:4">
+      <c r="A7212" t="s">
+        <v>7218</v>
+      </c>
+      <c r="D7212" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 77807b97ad3347b955bb44415ad5422fdfe21b5e 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/GLIDENumber.xlsx
+++ b/api/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14429" uniqueCount="7219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14433" uniqueCount="7221">
   <si>
     <t>code</t>
   </si>
@@ -41,6 +41,12 @@
   </si>
   <si>
     <t>en</t>
+  </si>
+  <si>
+    <t>EQ-2020-000241-HRV</t>
+  </si>
+  <si>
+    <t>FF-2020-000240-ZMB</t>
   </si>
   <si>
     <t>TC-2020-000239-MDG</t>
@@ -22002,7 +22008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7212"/>
+  <dimension ref="A1:G7214"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -79716,6 +79722,22 @@
         <v>8</v>
       </c>
     </row>
+    <row r="7213" spans="1:4">
+      <c r="A7213" t="s">
+        <v>7219</v>
+      </c>
+      <c r="D7213" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7214" spans="1:4">
+      <c r="A7214" t="s">
+        <v>7220</v>
+      </c>
+      <c r="D7214" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 27f377c33ab96b40e54d35bcaa293f70f1479ce5 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/GLIDENumber.xlsx
+++ b/api/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14437" uniqueCount="7223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14439" uniqueCount="7224">
   <si>
     <t>code</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>FL-2021-000001-MYS</t>
+  </si>
+  <si>
+    <t>CW-2020-000243-MNG</t>
   </si>
   <si>
     <t>FL-2020-000242-COL</t>
@@ -22014,7 +22017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7216"/>
+  <dimension ref="A1:G7217"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -79760,6 +79763,14 @@
         <v>8</v>
       </c>
     </row>
+    <row r="7217" spans="1:4">
+      <c r="A7217" t="s">
+        <v>7223</v>
+      </c>
+      <c r="D7217" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 45c40403c0b1a258e9a99a490d25b34eb4e2d74b 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/GLIDENumber.xlsx
+++ b/api/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14439" uniqueCount="7224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14441" uniqueCount="7225">
   <si>
     <t>code</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>en</t>
+  </si>
+  <si>
+    <t>CW-2021-000002-JPN</t>
   </si>
   <si>
     <t>FL-2021-000001-MYS</t>
@@ -22017,7 +22020,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7217"/>
+  <dimension ref="A1:G7218"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -79771,6 +79774,14 @@
         <v>8</v>
       </c>
     </row>
+    <row r="7218" spans="1:4">
+      <c r="A7218" t="s">
+        <v>7224</v>
+      </c>
+      <c r="D7218" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>